<commit_message>
fix: access m2Variedad by column name
</commit_message>
<xml_diff>
--- a/Produccion Astroflores BL25-26-27-28 a la Semana 21_entrenamiento.xlsx
+++ b/Produccion Astroflores BL25-26-27-28 a la Semana 21_entrenamiento.xlsx
@@ -4,19 +4,22 @@
   <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4507"/>
   <workbookPr defaultThemeVersion="124226"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="105" windowWidth="20115" windowHeight="7755"/>
+    <workbookView xWindow="9195" yWindow="-30" windowWidth="13815" windowHeight="7815"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
     <sheet name="Hoja2" sheetId="2" r:id="rId2"/>
     <sheet name="Hoja3" sheetId="3" r:id="rId3"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Hoja1!$A$1:$K$609</definedName>
+  </definedNames>
   <calcPr calcId="125725"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2443" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2475" uniqueCount="26">
   <si>
     <t>Anio</t>
   </si>
@@ -471,7 +474,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K609"/>
+  <dimension ref="A1:K617"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:11">
@@ -21854,7 +21857,7 @@
         <v>12800</v>
       </c>
       <c r="K578" s="6">
-        <f t="shared" ref="K578:K609" si="18">+H578/I578</f>
+        <f t="shared" ref="K578:K617" si="18">+H578/I578</f>
         <v>0.43864646234476468</v>
       </c>
     </row>
@@ -21878,7 +21881,7 @@
         <v>17</v>
       </c>
       <c r="G579" s="4" t="str">
-        <f t="shared" ref="G579:G609" si="19">+E579&amp;F579</f>
+        <f t="shared" ref="G579:G617" si="19">+E579&amp;F579</f>
         <v>025PINK MONDIAL</v>
       </c>
       <c r="H579" s="4">
@@ -23005,7 +23008,308 @@
         <v>0.82032585165774174</v>
       </c>
     </row>
+    <row r="610" spans="1:11">
+      <c r="A610" s="3">
+        <v>2026</v>
+      </c>
+      <c r="B610" s="4">
+        <v>26</v>
+      </c>
+      <c r="C610" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="D610" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="E610" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F610" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="G610" s="4" t="str">
+        <f t="shared" si="19"/>
+        <v>026PURPLE BUBBLY</v>
+      </c>
+      <c r="H610" s="4">
+        <v>740</v>
+      </c>
+      <c r="I610" s="4">
+        <v>1755.4</v>
+      </c>
+      <c r="J610" s="4">
+        <v>12800</v>
+      </c>
+      <c r="K610" s="6">
+        <f t="shared" si="18"/>
+        <v>0.42155634043522844</v>
+      </c>
+    </row>
+    <row r="611" spans="1:11">
+      <c r="A611" s="3">
+        <v>2026</v>
+      </c>
+      <c r="B611" s="4">
+        <v>26</v>
+      </c>
+      <c r="C611" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="D611" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="E611" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="F611" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="G611" s="4" t="str">
+        <f t="shared" si="19"/>
+        <v>025PINK MONDIAL</v>
+      </c>
+      <c r="H611" s="4">
+        <v>4425</v>
+      </c>
+      <c r="I611" s="4">
+        <v>3071.9505625000002</v>
+      </c>
+      <c r="J611" s="4">
+        <v>22400</v>
+      </c>
+      <c r="K611" s="6">
+        <f t="shared" si="18"/>
+        <v>1.4404528686161107</v>
+      </c>
+    </row>
+    <row r="612" spans="1:11">
+      <c r="A612" s="3">
+        <v>2026</v>
+      </c>
+      <c r="B612" s="4">
+        <v>26</v>
+      </c>
+      <c r="C612" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="D612" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="E612" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F612" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="G612" s="4" t="str">
+        <f t="shared" si="19"/>
+        <v>026LOLA</v>
+      </c>
+      <c r="H612" s="4">
+        <v>4325</v>
+      </c>
+      <c r="I612" s="4">
+        <v>1097.125</v>
+      </c>
+      <c r="J612" s="4">
+        <v>8000</v>
+      </c>
+      <c r="K612" s="6">
+        <f t="shared" si="18"/>
+        <v>3.9421214537997038</v>
+      </c>
+    </row>
+    <row r="613" spans="1:11">
+      <c r="A613" s="3">
+        <v>2026</v>
+      </c>
+      <c r="B613" s="4">
+        <v>26</v>
+      </c>
+      <c r="C613" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="D613" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="E613" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F613" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="G613" s="4" t="str">
+        <f t="shared" si="19"/>
+        <v>026PALOMA</v>
+      </c>
+      <c r="H613" s="4">
+        <v>4800</v>
+      </c>
+      <c r="I613" s="4">
+        <v>2852.5250000000001</v>
+      </c>
+      <c r="J613" s="4">
+        <v>20800</v>
+      </c>
+      <c r="K613" s="6">
+        <f t="shared" si="18"/>
+        <v>1.6827196957081882</v>
+      </c>
+    </row>
+    <row r="614" spans="1:11">
+      <c r="A614" s="3">
+        <v>2026</v>
+      </c>
+      <c r="B614" s="4">
+        <v>26</v>
+      </c>
+      <c r="C614" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="D614" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="E614" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="F614" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="G614" s="4" t="str">
+        <f t="shared" si="19"/>
+        <v>027SATISFACTION</v>
+      </c>
+      <c r="H614" s="4">
+        <v>2250</v>
+      </c>
+      <c r="I614" s="4">
+        <v>2633.1</v>
+      </c>
+      <c r="J614" s="4">
+        <v>19200</v>
+      </c>
+      <c r="K614" s="6">
+        <f t="shared" si="18"/>
+        <v>0.85450609547681444</v>
+      </c>
+    </row>
+    <row r="615" spans="1:11">
+      <c r="A615" s="3">
+        <v>2026</v>
+      </c>
+      <c r="B615" s="4">
+        <v>26</v>
+      </c>
+      <c r="C615" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="D615" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="E615" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="F615" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="G615" s="4" t="str">
+        <f t="shared" si="19"/>
+        <v>027TIFFANY!</v>
+      </c>
+      <c r="H615" s="4">
+        <v>2700</v>
+      </c>
+      <c r="I615" s="4">
+        <v>2633.1</v>
+      </c>
+      <c r="J615" s="4">
+        <v>19200</v>
+      </c>
+      <c r="K615" s="6">
+        <f t="shared" si="18"/>
+        <v>1.0254073145721774</v>
+      </c>
+    </row>
+    <row r="616" spans="1:11">
+      <c r="A616" s="3">
+        <v>2026</v>
+      </c>
+      <c r="B616" s="4">
+        <v>26</v>
+      </c>
+      <c r="C616" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="D616" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="E616" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="F616" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="G616" s="4" t="str">
+        <f t="shared" si="19"/>
+        <v>028COTOPAXI</v>
+      </c>
+      <c r="H616" s="4">
+        <v>2670</v>
+      </c>
+      <c r="I616" s="4">
+        <v>2852.5250000000001</v>
+      </c>
+      <c r="J616" s="4">
+        <v>20800</v>
+      </c>
+      <c r="K616" s="6">
+        <f t="shared" si="18"/>
+        <v>0.93601283073767971</v>
+      </c>
+    </row>
+    <row r="617" spans="1:11">
+      <c r="A617" s="3">
+        <v>2026</v>
+      </c>
+      <c r="B617" s="4">
+        <v>26</v>
+      </c>
+      <c r="C617" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="D617" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="E617" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="F617" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="G617" s="4" t="str">
+        <f t="shared" si="19"/>
+        <v>028DEEP PURPLE</v>
+      </c>
+      <c r="H617" s="4">
+        <v>3420</v>
+      </c>
+      <c r="I617" s="4">
+        <v>2852.5250000000001</v>
+      </c>
+      <c r="J617" s="4">
+        <v>20800</v>
+      </c>
+      <c r="K617" s="6">
+        <f t="shared" si="18"/>
+        <v>1.1989377831920842</v>
+      </c>
+    </row>
   </sheetData>
+  <autoFilter ref="A1:K609">
+    <filterColumn colId="0"/>
+    <filterColumn colId="1"/>
+    <filterColumn colId="5"/>
+  </autoFilter>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>

</xml_diff>